<commit_message>
backlog en user stories bijna klaar
</commit_message>
<xml_diff>
--- a/backlog project.xlsx
+++ b/backlog project.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ehb-my.sharepoint.com/personal/lilian_levano_student_ehb_be/Documents/école ehb/cours/dynamic web prg1 s2/ExamenProject/Project-Dynamic-Web/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="91" documentId="11_F25DC773A252ABDACC10483A31DF42745BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24067FB8-9E2F-4F97-8E28-D3F664A41BA6}"/>
+  <xr:revisionPtr revIDLastSave="127" documentId="11_F25DC773A252ABDACC10483A31DF42745BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69861217-FEA4-43DE-8098-C75E281C0B4A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="33">
   <si>
     <t>TaskID</t>
   </si>
@@ -71,58 +71,105 @@
     <t>Als een user die de website bezoekt, wil ik een lijst van alle historische locaties in Brussel in een tabel met minimum 6 kolommen van informatie, zodat ik me kan informeren over alle beschikbare historische locaties in Brussel.</t>
   </si>
   <si>
-    <t>Bij het opstarten van het website wordt een functie fetchData() opgeroept om de API aan te spreken, en via een functie updateMainList() de effectieve lijst van locaties te maken / aan te passen.</t>
-  </si>
-  <si>
-    <t>De url moet effectief naar de API die de dataset van de historische locaties bevat verwijzen zonder fouten.</t>
-  </si>
-  <si>
-    <t>Elk user dat voor het eerst de website bezoekt moet een default waarde krijgen voor elke mogelijke key in de localStorage, bijvoorbeeld "nl" bij "taal".</t>
-  </si>
-  <si>
     <t>In de CSS file verschillende media querries aanmaken die ervoor zorgen dat de website op elke mogelijke device bruikbaar is.</t>
   </si>
   <si>
-    <t>De website moet zich aanpassen volgens deze verschillende schermgroottes:
-…</t>
-  </si>
-  <si>
     <t xml:space="preserve">Als een user die de website bezoekt, wil ik de mogelijkheid hebben om de lijst van historische locaties in Brussel te filtreren (op type, locatie, etc…), zodat ik mijn lijst kan beperken tot de gemeente dat ik nodig heb. </t>
   </si>
   <si>
     <t>Als een user die de website bezoekt, wil ik de mogelijkheid hebben om een specifieke locatie op te zoeken, zodat ik op een snelle manier een locatie kan vinden.</t>
   </si>
   <si>
-    <t>Door op de knop "search" te drukken, opent een cover, waarin alle locaties worden opgelijst. Een user kan dan intypen in het balk bovenaan om een specifieke locatie op naam op te zoeken.</t>
-  </si>
-  <si>
-    <t>Om een locatie op te zoeken, moet de user het zoeken op basis van de naam van de locatie. Minstens één locatie met deze naam moet bestaan om een lijst te krijgen, anders wordt een bericht getoond die hem waarschuwt dat er geen locatie die corresponderen.</t>
-  </si>
-  <si>
     <t>Als een user die de website bezoekt, wil ik de mogelijkheid hebben om de lijst op de homepage te sorteren, zodat ik de locaties kan zien in de volgorde dat ik wil.</t>
   </si>
   <si>
-    <t xml:space="preserve">Wanneer een post-code wordt ingevoerd in de input voor de post-code, worden alle elementen met die zelfde post-code samengenomen en getoond in de lijst. 
+    <t>Sorteermethode…</t>
+  </si>
+  <si>
+    <t>Als een user die de website bezoekt, wil ik de mogelijkheid om bepaalde voorkeuren (bijvoorbeeld: mijn taal) te veranderen en die op te slagen doorheen verschillende sessies.</t>
+  </si>
+  <si>
+    <t>Als een user die de website bezoekt, wil ik bepaalde locaties als favoriet kunnen opslaan, waarbij deze locatie wordt bijgehouden tussen mijn sessies, zodat ik snel mijn locaties kan terug vinden.</t>
+  </si>
+  <si>
+    <t>Als een user die de website bezoekt, wil ik een duidelijke een aantrekkelijke UI, waarvan de button duidelijk aantonen wat hun functies zijn, zodat ik de website op een efficiënte manier kan gebruiken.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">De website toont een lijst van historische locaties in een tabel
+De tabel bevat minstens 6 kolommen met relevante informatie
+De data wordt correct opgehaald via de API
+Bij een fout in de fetch wordt een foutmelding getoond
 </t>
   </si>
   <si>
-    <t>Sorteermethode…</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Om te filtreren moet de user effectief een post-code, een nummer dus, invoeren. Minstens één locatie met die post-code moet bestaan om effectief een lijst te zien, anders wordt een bericht getoond die hem waarschuwt dat er geen locatie die corresponderen.
+    <t xml:space="preserve">De gebruiker kan filteren op minstens één criterium (bv. type of locatie)
+De lijst past zich aan wanneer de user op de filtreer button klikt, op basis van de gekozen filters
+Enkel overeenkomende resultaten worden weergegeven
+Bij geen resultaten wordt een duidelijke melding getoond
+De gebruiker kan filters resetten, wat alle locaties opnieuw toont
 </t>
   </si>
   <si>
-    <t>Als een user die de website bezoekt, wil ik de mogelijkheid om bepaalde voorkeuren (bijvoorbeeld: mijn taal) te veranderen en die op te slagen doorheen verschillende sessies.</t>
-  </si>
-  <si>
-    <t>Twee buttons aanmaken om de taal van de user te switchen. Wanneer een button gedrukt werd, herlaad de hele website volgens de gekoze taal en wordt de taal opgeslagen in de localStorage van de user.</t>
-  </si>
-  <si>
-    <t>Een user kan door een klein knopje een locatie als favoriet kiezen, en kan deze zien in het menu van favoriete locaties. Een favoriete locatie wordt bijgehouden in een array, onder de key (favorites) in de localStorage van de user.</t>
-  </si>
-  <si>
-    <t>Als een user die de website bezoekt, wil ik bepaalde locaties als favoriet kunnen opslaan, waarbij deze locaties wordt bijgehouden tussen mijn sessies, zodat ik snel mijn locaties kan terug vinden.</t>
+    <t>De gebruiker kan zoeken op naam van een locatie
+De lijst wordt live aangepast tijdens het typen
+Bij een lege zoekopdracht wordt de volledige lijst getoond
+Bij geen resultaten wordt een melding weergegeven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">De gebruiker kan de lijst sorteren volgens minstens één criterium
+De sortering wordt correct toegepast op de volledige lijst
+De lijst wordt visueel aangepast na sortering
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">De gebruiker kan locaties toevoegen aan favorieten
+Favorieten worden opgeslagen in LocalStorage
+Favorieten blijven bewaard tussen sessies
+Dubbele favorieten worden niet toegestaan
+</t>
+  </si>
+  <si>
+    <t>De gebruiker kan een taalvoorkeur selecteren
+De gekozen taal wordt opgeslagen in LocalStorage
+De taal wordt automatisch toegepast bij herladen van de website
+Een standaardtaal wordt ingesteld bij eerste bezoek</t>
+  </si>
+  <si>
+    <t>De website werkt op verschillende schermgroottes
+De layout past zich automatisch aan (desktop, tablet, mobiel)
+Elementen blijven leesbaar en bruikbaar op alle devices
+Geen functionaliteit gaat verloren bij kleinere schermen</t>
+  </si>
+  <si>
+    <t>De interface is overzichtelijk en consistent
+Knoppen zijn duidelijk herkenbaar en begrijpelijk
+Interactieve elementen geven visuele feedback
+Navigatie is intuïtief en gebruiksvriendelijk</t>
+  </si>
+  <si>
+    <t>Maak een functie fetchData met als parameters withAllLanguage om eerst een array te maken met alle mogelijke locaties, dan kan fetchData zonder parameters gebruikt worden om per taal de locaties te tonen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maak een filtreer button waaraan we een EventListener toevoegen
+Wanneer die button geklikt wordt, neemt het de value van de input voor de post code en past de main list eraan toe.
+Er moet ook gechekt worden of de input effectief een belgische post code kan zijn, dus maximaal en minimaal 4 digits
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maak een search button en voeg er een EventListeren toe. Wanneer de button geklikt wordt, wordt er een  nieuwe cover opnieuw gemaakt.
+In de cover wordt een nieuwe lijst aangemaakt met alle mogelijke locaties, waarvan de taal veranderd wegens een check op voorhand op de localStorage.
+Een balk wordt toegevoegd, waaraan een EventListener elke input detecteert, en bij elke input wordt er gechekt of er locaties zijn die corresponderen met wat er in de balk werd ingevoerd.  </t>
+  </si>
+  <si>
+    <t>Voor elke kaart, voeg een SVG die de ID van de locatie overneemt en een EventListener heeft. Als de SVG geklikt wordt, wordt er met .find() een relatie gezocht tussen de ID van de SVG en die in de eerste array van locaties dat we maken. Dit zal ervoor zorgen dat we de object kunnen nemen van de locatie, en zo de data op een efficiente manier kan gebruiken om die in de array van favoriete locaties pushen in de localStorage van de user.
+Via een knop kan de user een menu openen dat al zijn favoriete locaties oplijst, en kan deze ook verwijderen van zijn lijst.</t>
+  </si>
+  <si>
+    <t>Twee buttons aanmaken om de taal van de user te switchen. Wanneer een button gedrukt werd, herlaad de hele website volgens de gekoze taal en wordt de taal opgeslagen in de localStorage van de user.
+Bij het opladen van de website wordt er een check gedaan om de taal van de website aan te passen.</t>
+  </si>
+  <si>
+    <t>Duidelijke icoontjes en tekst gebruiken om ervoor te zorgen dat de website duidelijke en gebruikersvriendelijk is.</t>
   </si>
 </sst>
 </file>
@@ -483,9 +530,9 @@
   <dimension ref="B2:H10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="62.140625" customWidth="1"/>
-    <col min="6" max="6" width="97" customWidth="1"/>
-    <col min="7" max="7" width="110.7109375" customWidth="1"/>
+    <col min="5" max="5" width="44.85546875" customWidth="1"/>
+    <col min="6" max="6" width="51.28515625" customWidth="1"/>
+    <col min="7" max="7" width="64" customWidth="1"/>
     <col min="8" max="8" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -526,10 +573,10 @@
         <v>10</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>8</v>
@@ -546,13 +593,13 @@
         <v>7</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>8</v>
@@ -569,15 +616,17 @@
         <v>7</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5" s="2"/>
+        <v>21</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="6" spans="2:8" ht="246" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="2">
@@ -590,19 +639,21 @@
         <v>7</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H6" s="2"/>
+      <c r="H6" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="7" spans="2:8" ht="297.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C7" s="2">
         <v>1</v>
@@ -611,34 +662,44 @@
         <v>7</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="2:8" ht="297.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
+      <c r="B8" s="2">
+        <v>6</v>
+      </c>
+      <c r="C8" s="2">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="E8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
+      <c r="H8" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="9" spans="2:8" ht="183" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="2">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C9" s="2">
         <v>1</v>
@@ -650,23 +711,37 @@
         <v>9</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="135.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
+      <c r="B10" s="2">
+        <v>8</v>
+      </c>
+      <c r="C10" s="2">
+        <v>1</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
backlog / US pdf
</commit_message>
<xml_diff>
--- a/backlog project.xlsx
+++ b/backlog project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ehb-my.sharepoint.com/personal/lilian_levano_student_ehb_be/Documents/école ehb/cours/dynamic web prg1 s2/ExamenProject/Project-Dynamic-Web/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{569204C9-D857-4574-B249-9033F4B542D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6B0F070-77B2-4D06-A77B-A6FAAF4A9A61}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{569204C9-D857-4574-B249-9033F4B542D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AFB3B6C2-67C0-4CAE-9346-0D9BD762F595}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -761,7 +761,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="8" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>